<commit_message>
add youtube_fetcher.py, integrate YT data into run.py
</commit_message>
<xml_diff>
--- a/MKTBrs_競品分析工作包.xlsx
+++ b/MKTBrs_競品分析工作包.xlsx
@@ -1048,18 +1048,26 @@
         <f>IFERROR((N3+O3)/J3,"–")</f>
         <v/>
       </c>
-      <c r="Q3" s="19" t="n"/>
-      <c r="R3" s="19" t="n"/>
-      <c r="S3" s="19" t="n"/>
-      <c r="T3" s="20">
-        <f>IFERROR(S3/R3,"–")</f>
-        <v/>
-      </c>
-      <c r="U3" s="19" t="n"/>
-      <c r="V3" s="19" t="n"/>
-      <c r="W3" s="20">
-        <f>IFERROR(V3/U3,"–")</f>
-        <v/>
+      <c r="Q3" s="19" t="n">
+        <v>23100</v>
+      </c>
+      <c r="R3" s="19" t="n">
+        <v>1171</v>
+      </c>
+      <c r="S3" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="19" t="n">
+        <v>222852</v>
+      </c>
+      <c r="V3" s="19" t="n">
+        <v>2976</v>
+      </c>
+      <c r="W3" s="20" t="n">
+        <v>0.0134</v>
       </c>
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="n"/>
@@ -1103,18 +1111,26 @@
         <f>IFERROR((N4+O4)/J4,"–")</f>
         <v/>
       </c>
-      <c r="Q4" s="21" t="n"/>
-      <c r="R4" s="21" t="n"/>
-      <c r="S4" s="21" t="n"/>
-      <c r="T4" s="22">
-        <f>IFERROR(S4/R4,"–")</f>
-        <v/>
-      </c>
-      <c r="U4" s="21" t="n"/>
-      <c r="V4" s="21" t="n"/>
-      <c r="W4" s="22">
-        <f>IFERROR(V4/U4,"–")</f>
-        <v/>
+      <c r="Q4" s="21" t="n">
+        <v>861</v>
+      </c>
+      <c r="R4" s="21" t="n">
+        <v>1530</v>
+      </c>
+      <c r="S4" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="T4" s="22" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="U4" s="21" t="n">
+        <v>1530</v>
+      </c>
+      <c r="V4" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="W4" s="22" t="n">
+        <v>0.0111</v>
       </c>
       <c r="X4" s="5" t="n"/>
       <c r="Y4" s="5" t="n"/>
@@ -1158,18 +1174,26 @@
         <f>IFERROR((N5+O5)/J5,"–")</f>
         <v/>
       </c>
-      <c r="Q5" s="19" t="n"/>
-      <c r="R5" s="19" t="n"/>
-      <c r="S5" s="19" t="n"/>
-      <c r="T5" s="20">
-        <f>IFERROR(S5/R5,"–")</f>
-        <v/>
-      </c>
-      <c r="U5" s="19" t="n"/>
-      <c r="V5" s="19" t="n"/>
-      <c r="W5" s="20">
-        <f>IFERROR(V5/U5,"–")</f>
-        <v/>
+      <c r="Q5" s="19" t="n">
+        <v>96</v>
+      </c>
+      <c r="R5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="X5" s="2" t="n"/>
       <c r="Y5" s="2" t="n"/>
@@ -1213,18 +1237,26 @@
         <f>IFERROR((N6+O6)/J6,"–")</f>
         <v/>
       </c>
-      <c r="Q6" s="21" t="n"/>
-      <c r="R6" s="21" t="n"/>
-      <c r="S6" s="21" t="n"/>
-      <c r="T6" s="22">
-        <f>IFERROR(S6/R6,"–")</f>
-        <v/>
-      </c>
-      <c r="U6" s="21" t="n"/>
-      <c r="V6" s="21" t="n"/>
-      <c r="W6" s="22">
-        <f>IFERROR(V6/U6,"–")</f>
-        <v/>
+      <c r="Q6" s="21" t="n">
+        <v>270</v>
+      </c>
+      <c r="R6" s="21" t="n">
+        <v>917</v>
+      </c>
+      <c r="S6" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="22" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="U6" s="21" t="n">
+        <v>6745</v>
+      </c>
+      <c r="V6" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="W6" s="22" t="n">
+        <v>0.0021</v>
       </c>
       <c r="X6" s="5" t="n"/>
       <c r="Y6" s="5" t="n"/>
@@ -1268,18 +1300,26 @@
         <f>IFERROR((N7+O7)/J7,"–")</f>
         <v/>
       </c>
-      <c r="Q7" s="19" t="n"/>
-      <c r="R7" s="19" t="n"/>
-      <c r="S7" s="19" t="n"/>
-      <c r="T7" s="20">
-        <f>IFERROR(S7/R7,"–")</f>
-        <v/>
-      </c>
-      <c r="U7" s="19" t="n"/>
-      <c r="V7" s="19" t="n"/>
-      <c r="W7" s="20">
-        <f>IFERROR(V7/U7,"–")</f>
-        <v/>
+      <c r="Q7" s="19" t="n">
+        <v>74200</v>
+      </c>
+      <c r="R7" s="19" t="n">
+        <v>19012</v>
+      </c>
+      <c r="S7" s="19" t="n">
+        <v>230</v>
+      </c>
+      <c r="T7" s="20" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="U7" s="19" t="n">
+        <v>320599</v>
+      </c>
+      <c r="V7" s="19" t="n">
+        <v>2897</v>
+      </c>
+      <c r="W7" s="20" t="n">
+        <v>0.008999999999999999</v>
       </c>
       <c r="X7" s="2" t="n"/>
       <c r="Y7" s="2" t="n"/>

</xml_diff>

<commit_message>
add social_input.py with 10-post entry and frequency calculation
</commit_message>
<xml_diff>
--- a/MKTBrs_競品分析工作包.xlsx
+++ b/MKTBrs_競品分析工作包.xlsx
@@ -168,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -234,6 +234,8 @@
     <xf numFmtId="10" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -779,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AC7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -817,48 +819,53 @@
           <t>基本資料</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
+      <c r="B1" s="23" t="n"/>
       <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="D1" s="9" t="n"/>
-      <c r="E1" s="9" t="n"/>
-      <c r="F1" s="9" t="n"/>
-      <c r="G1" s="9" t="n"/>
-      <c r="H1" s="9" t="n"/>
-      <c r="I1" s="9" t="n"/>
+      <c r="D1" s="24" t="n"/>
+      <c r="E1" s="24" t="n"/>
+      <c r="F1" s="24" t="n"/>
+      <c r="G1" s="24" t="n"/>
+      <c r="H1" s="24" t="n"/>
+      <c r="I1" s="23" t="n"/>
       <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K1" s="9" t="n"/>
-      <c r="L1" s="9" t="n"/>
-      <c r="M1" s="9" t="n"/>
-      <c r="N1" s="9" t="n"/>
-      <c r="O1" s="9" t="n"/>
-      <c r="P1" s="9" t="n"/>
+      <c r="K1" s="24" t="n"/>
+      <c r="L1" s="24" t="n"/>
+      <c r="M1" s="24" t="n"/>
+      <c r="N1" s="24" t="n"/>
+      <c r="O1" s="24" t="n"/>
+      <c r="P1" s="23" t="n"/>
       <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="R1" s="9" t="n"/>
-      <c r="S1" s="9" t="n"/>
-      <c r="T1" s="9" t="n"/>
-      <c r="U1" s="9" t="n"/>
-      <c r="V1" s="9" t="n"/>
-      <c r="W1" s="9" t="n"/>
+      <c r="R1" s="24" t="n"/>
+      <c r="S1" s="24" t="n"/>
+      <c r="T1" s="24" t="n"/>
+      <c r="U1" s="24" t="n"/>
+      <c r="V1" s="24" t="n"/>
+      <c r="W1" s="23" t="n"/>
       <c r="X1" s="13" t="inlineStr">
         <is>
           <t>商業規模</t>
         </is>
       </c>
-      <c r="Y1" s="9" t="n"/>
-      <c r="Z1" s="9" t="n"/>
-      <c r="AA1" s="9" t="n"/>
+      <c r="Y1" s="24" t="n"/>
+      <c r="Z1" s="24" t="n"/>
+      <c r="AA1" s="23" t="n"/>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>發文頻率</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
@@ -1010,6 +1017,16 @@
           <t>備註</t>
         </is>
       </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>FB 發文頻率</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>IG 發文頻率</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1022,9 +1039,15 @@
           <t>https://dio3212.kaik.io</t>
         </is>
       </c>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="19" t="n"/>
-      <c r="E3" s="19" t="n"/>
+      <c r="C3" s="19" t="n">
+        <v>123</v>
+      </c>
+      <c r="D3" s="19" t="n">
+        <v>20240323</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>111</v>
+      </c>
       <c r="F3" s="20">
         <f>IFERROR((D3+E3)/C3,"–")</f>
         <v/>
@@ -1329,9 +1352,9 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="J1:P1"/>
+    <mergeCell ref="C1:I1"/>
     <mergeCell ref="Q1:W1"/>
     <mergeCell ref="X1:AA1"/>
-    <mergeCell ref="C1:I1"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>